<commit_message>
updated implementations of scoring strategies
</commit_message>
<xml_diff>
--- a/data/raw/metamethod review/codebook - rater 1 - original/calc_strat_revised.xlsx
+++ b/data/raw/metamethod review/codebook - rater 1 - original/calc_strat_revised.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10911"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/Dropbox/Academic work/RUB &amp; HTI work/Supervision/Annika's BA thesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/git/igt-project/data/raw/metamethod review/codebook - rater 1 - original/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82657B2A-722E-C845-AB0B-5CC9457362A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E732EC-A5A3-CA4D-8B79-436735224DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="26380" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="351">
   <si>
     <t>strategy_id</t>
   </si>
@@ -1035,6 +1035,60 @@
   </si>
   <si>
     <t>isn't this equivalent to the previous one? There's a fixed number of trials, so dividing by N trials is a monotonic transformation.</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>implemented_in_multiverse</t>
+  </si>
+  <si>
+    <t>isn't this monotonic with strategy ignoring captial? What value to use for starting capital?</t>
+  </si>
+  <si>
+    <t>if interpretation of above metric is correct, this should be 1-(that value). Ie the strategies are monotonicly identical.</t>
+  </si>
+  <si>
+    <t>same as previous one?</t>
+  </si>
+  <si>
+    <t>is this related to the previous two?</t>
+  </si>
+  <si>
+    <t>switching</t>
+  </si>
+  <si>
+    <t>switching after loss</t>
+  </si>
+  <si>
+    <t>non switching after loss on A</t>
+  </si>
+  <si>
+    <t>switching after loss on A or B to C or D after a loss on A or B</t>
+  </si>
+  <si>
+    <t>(DIS)ADVANTAGEOUS CHOICES (WIN/LOSS DICHOTOMISED)</t>
+  </si>
+  <si>
+    <t>COUNTS OF DECK SELECTIONS</t>
+  </si>
+  <si>
+    <t>(POST LOSS) DECK SWIT CHING</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>MONETARY CONSEQUENCES</t>
+  </si>
+  <si>
+    <t>??? Isn't this the same as total balance ignoring the first trial?</t>
+  </si>
+  <si>
+    <t>as in count of card selections where the money won - money lost is &gt;0? Or count of cards where win was 100 instead of just 50?</t>
   </si>
 </sst>
 </file>
@@ -1160,7 +1214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1280,20 +1334,149 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3546,305 +3729,465 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F455A80B-30A2-1B4E-B1CF-4FD357DAC636}">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.5" customWidth="1"/>
-    <col min="2" max="2" width="43.33203125" style="23" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" style="44" customWidth="1"/>
+    <col min="1" max="1" width="31.83203125" style="49" customWidth="1"/>
+    <col min="2" max="2" width="43.33203125" style="50" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" style="94" customWidth="1"/>
+    <col min="4" max="4" width="24" style="49" customWidth="1"/>
+    <col min="5" max="5" width="51.33203125" style="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="47" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="D1" s="49" t="s">
+        <v>335</v>
+      </c>
+      <c r="E1" s="50" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="51"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="54"/>
+    </row>
+    <row r="3" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="55" t="s">
+        <v>348</v>
+      </c>
+      <c r="B3" s="52"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="54"/>
+    </row>
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B4" s="57" t="s">
         <v>101</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C4" s="58" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="E4" s="50" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B5" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C5" s="58" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="D5" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B6" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C6" s="58" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="D6" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B7" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C7" s="58" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="D7" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="59"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="54"/>
+    </row>
+    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="61" t="s">
+        <v>344</v>
+      </c>
+      <c r="B9" s="60"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="53"/>
+      <c r="E9" s="54"/>
+    </row>
+    <row r="10" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A10" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B10" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C10" s="58" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="E10" s="50" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A11" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B11" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C11" s="58" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="E11" s="50" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A12" s="62" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="C12" s="64"/>
+      <c r="E12" s="50" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A13" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B13" s="57" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C13" s="58" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="E13" s="50" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="59"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="54"/>
+    </row>
+    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="61" t="s">
+        <v>345</v>
+      </c>
+      <c r="B15" s="60"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="54"/>
+    </row>
+    <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="65" t="s">
         <v>325</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B16" s="66" t="s">
         <v>144</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C16" s="67" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="D16" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="68" t="s">
+        <v>328</v>
+      </c>
+      <c r="B17" s="69" t="s">
+        <v>194</v>
+      </c>
+      <c r="C17" s="70" t="s">
+        <v>329</v>
+      </c>
+      <c r="D17" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="68" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="69" t="s">
+        <v>152</v>
+      </c>
+      <c r="C18" s="70" t="s">
+        <v>200</v>
+      </c>
+      <c r="D18" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="68" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="69" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" s="70" t="s">
+        <v>326</v>
+      </c>
+      <c r="D19" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A20" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="64" t="s">
+        <v>245</v>
+      </c>
+      <c r="D20" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="68" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="69" t="s">
+        <v>154</v>
+      </c>
+      <c r="C21" s="70" t="s">
+        <v>327</v>
+      </c>
+      <c r="D21" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A22" s="62" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="63" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="64" t="s">
+        <v>246</v>
+      </c>
+      <c r="D22" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A23" s="71" t="s">
+        <v>331</v>
+      </c>
+      <c r="B23" s="72" t="s">
+        <v>156</v>
+      </c>
+      <c r="C23" s="73" t="s">
+        <v>330</v>
+      </c>
+      <c r="D23" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A24" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="B24" s="72" t="s">
+        <v>205</v>
+      </c>
+      <c r="C24" s="75" t="s">
+        <v>322</v>
+      </c>
+      <c r="E24" s="50" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="76" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="78" t="s">
+        <v>247</v>
+      </c>
+      <c r="D25" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A26" s="62" t="s">
+        <v>320</v>
+      </c>
+      <c r="B26" s="63" t="s">
+        <v>318</v>
+      </c>
+      <c r="C26" s="79" t="s">
+        <v>319</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="80" t="s">
+        <v>317</v>
+      </c>
+      <c r="B27" s="81" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="82" t="s">
+        <v>315</v>
+      </c>
+      <c r="D27" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A28" s="83" t="s">
+        <v>321</v>
+      </c>
+      <c r="B28" s="63" t="s">
+        <v>187</v>
+      </c>
+      <c r="C28" s="79" t="s">
+        <v>316</v>
+      </c>
+      <c r="D28" s="49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="84"/>
+      <c r="B29" s="60"/>
+      <c r="C29" s="85"/>
+      <c r="D29" s="53"/>
+      <c r="E29" s="54"/>
+    </row>
+    <row r="30" spans="1:5" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="85" t="s">
+        <v>346</v>
+      </c>
+      <c r="B30" s="60"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="54"/>
+    </row>
+    <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="86" t="s">
+        <v>269</v>
+      </c>
+      <c r="B31" s="87" t="s">
+        <v>190</v>
+      </c>
+      <c r="C31" s="88"/>
+      <c r="E31" s="50" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="86" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" s="87" t="s">
+        <v>192</v>
+      </c>
+      <c r="C32" s="88"/>
+      <c r="E32" s="50" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A33" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B33" s="69" t="s">
         <v>150</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C33" s="70" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="39" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="C15" s="36" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A17" s="50" t="s">
-        <v>331</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="C17" s="51" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="B18" s="27" t="s">
-        <v>205</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>322</v>
-      </c>
-      <c r="D18" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="C19" s="40" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A20" s="49" t="s">
-        <v>317</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>164</v>
-      </c>
-      <c r="C20" s="38" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="64" x14ac:dyDescent="0.2">
-      <c r="A21" s="48" t="s">
-        <v>321</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="C21" s="47" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>318</v>
-      </c>
-      <c r="C22" s="47" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="48" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>184</v>
-      </c>
-      <c r="C23" s="39"/>
-    </row>
-    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="B24" s="31" t="s">
-        <v>190</v>
-      </c>
-      <c r="C24" s="41"/>
-    </row>
-    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="C25" s="41"/>
-    </row>
-    <row r="26" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A26" s="8" t="s">
+      <c r="E33" s="50" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A34" s="86" t="s">
         <v>69</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B34" s="87" t="s">
         <v>299</v>
       </c>
-      <c r="C26" s="42"/>
-    </row>
-    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="46" t="s">
+      <c r="C34" s="89"/>
+      <c r="E34" s="50" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="59"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="54"/>
+    </row>
+    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="61" t="s">
+        <v>347</v>
+      </c>
+      <c r="B36" s="60"/>
+      <c r="C36" s="90"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="54"/>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="91" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B37" s="92" t="s">
         <v>93</v>
       </c>
-      <c r="C27" s="43"/>
-      <c r="D27" t="s">
-        <v>303</v>
+      <c r="C37" s="93"/>
+      <c r="E37" s="50" t="s">
+        <v>333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>